<commit_message>
Fixed graph overlapping with text and added sum formulats to pivot table
</commit_message>
<xml_diff>
--- a/Automate_Excel_Report/pivot_table.xlsx
+++ b/Automate_Excel_Report/pivot_table.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;R&quot;#,##0"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -142,6 +145,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -152,7 +156,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Report'!B5</f>
+              <f>'Report'!B3</f>
             </strRef>
           </tx>
           <spPr>
@@ -162,12 +166,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$6:$A$7</f>
+              <f>'Report'!$A$4:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$B$6:$B$7</f>
+              <f>'Report'!$B$4:$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -176,7 +180,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Report'!C5</f>
+              <f>'Report'!C3</f>
             </strRef>
           </tx>
           <spPr>
@@ -186,12 +190,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$6:$A$7</f>
+              <f>'Report'!$A$4:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$C$6:$C$7</f>
+              <f>'Report'!$C$4:$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -200,7 +204,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Report'!D5</f>
+              <f>'Report'!D3</f>
             </strRef>
           </tx>
           <spPr>
@@ -210,12 +214,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$6:$A$7</f>
+              <f>'Report'!$A$4:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$D$6:$D$7</f>
+              <f>'Report'!$D$4:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -224,7 +228,7 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Report'!E5</f>
+              <f>'Report'!E3</f>
             </strRef>
           </tx>
           <spPr>
@@ -234,12 +238,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$6:$A$7</f>
+              <f>'Report'!$A$4:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$E$6:$E$7</f>
+              <f>'Report'!$E$4:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -248,7 +252,7 @@
           <order val="4"/>
           <tx>
             <strRef>
-              <f>'Report'!F5</f>
+              <f>'Report'!F3</f>
             </strRef>
           </tx>
           <spPr>
@@ -258,12 +262,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$6:$A$7</f>
+              <f>'Report'!$A$4:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$F$6:$F$7</f>
+              <f>'Report'!$F$4:$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -272,7 +276,7 @@
           <order val="5"/>
           <tx>
             <strRef>
-              <f>'Report'!G5</f>
+              <f>'Report'!G3</f>
             </strRef>
           </tx>
           <spPr>
@@ -282,12 +286,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Report'!$A$6:$A$7</f>
+              <f>'Report'!$A$4:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Report'!$G$6:$G$7</f>
+              <f>'Report'!$G$4:$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -320,6 +324,7 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -333,7 +338,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>9</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="2700000"/>
@@ -643,94 +648,120 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A5:G7"/>
+  <dimension ref="A3:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Electronic accessories</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Fashion accessories</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Food and beverages</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Health and beauty</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Home and lifestyle</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Sports and travel</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>27102</v>
+      </c>
+      <c r="C4" t="n">
+        <v>30437</v>
+      </c>
+      <c r="D4" t="n">
+        <v>33171</v>
+      </c>
+      <c r="E4" t="n">
+        <v>18561</v>
+      </c>
+      <c r="F4" t="n">
+        <v>30037</v>
+      </c>
+      <c r="G4" t="n">
+        <v>28575</v>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gender</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Electronic accessories</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Fashion accessories</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Food and beverages</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Health and beauty</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Home and lifestyle</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Sports and travel</t>
-        </is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>27236</v>
+      </c>
+      <c r="C5" t="n">
+        <v>23868</v>
+      </c>
+      <c r="D5" t="n">
+        <v>22974</v>
+      </c>
+      <c r="E5" t="n">
+        <v>30633</v>
+      </c>
+      <c r="F5" t="n">
+        <v>23825</v>
+      </c>
+      <c r="G5" t="n">
+        <v>26548</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>27102</v>
-      </c>
-      <c r="C6" t="n">
-        <v>30437</v>
-      </c>
-      <c r="D6" t="n">
-        <v>33171</v>
-      </c>
-      <c r="E6" t="n">
-        <v>18561</v>
-      </c>
-      <c r="F6" t="n">
-        <v>30037</v>
-      </c>
-      <c r="G6" t="n">
-        <v>28575</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>27236</v>
-      </c>
-      <c r="C7" t="n">
-        <v>23868</v>
-      </c>
-      <c r="D7" t="n">
-        <v>22974</v>
-      </c>
-      <c r="E7" t="n">
-        <v>30633</v>
-      </c>
-      <c r="F7" t="n">
-        <v>23825</v>
-      </c>
-      <c r="G7" t="n">
-        <v>26548</v>
+      <c r="B6" s="1">
+        <f>SUM(B4:B5)</f>
+        <v/>
+      </c>
+      <c r="C6" s="1">
+        <f>SUM(C4:C5)</f>
+        <v/>
+      </c>
+      <c r="D6" s="1">
+        <f>SUM(D4:D5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="1">
+        <f>SUM(E4:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="1">
+        <f>SUM(F4:F5)</f>
+        <v/>
+      </c>
+      <c r="G6" s="1">
+        <f>SUM(G4:G5)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>